<commit_message>
ODDS: surface real cash generated (+17.9M) instead of hiding in plug
По замечанию: остаток 0 вводил в заблуждение. Добавлен явный подытог
«ЧИСТЫЙ ДЕНЕЖНЫЙ ПОТОК ЗА ПЕРИОД (заработано деньгами) = +17,9 млн ₸».
Эти деньги размещены на депозит/прочие счета Группы (вне 5 выписок),
поэтому расчётные счета закрылись в 0. Показатель вынесен на дашборд.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QEQJkD5wucj2vbcLQp61wc
</commit_message>
<xml_diff>
--- a/waystar-management-report/WayStar_Управленка_Июль2026.xlsx
+++ b/waystar-management-report/WayStar_Управленка_Июль2026.xlsx
@@ -913,7 +913,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Операционный ден. поток</t>
+          <t>Заработано деньгами за месяц</t>
         </is>
       </c>
       <c r="B9" s="5" t="n"/>
@@ -931,8 +931,8 @@
       <c r="F9" s="5" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="6">
-        <f>'ОДДС'!C13</f>
+      <c r="A10" s="8">
+        <f>'ОДДС'!C31</f>
         <v/>
       </c>
       <c r="B10" s="7" t="n"/>
@@ -950,7 +950,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>от операц. деятельности</t>
+          <t>на депозите/прочих счетах Группы</t>
         </is>
       </c>
       <c r="B11" s="10" t="n"/>
@@ -1599,7 +1599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -1916,54 +1916,65 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="30" t="inlineStr">
-        <is>
-          <t>Перемещения на прочие счета Группы + конвертация валют (нетто)</t>
-        </is>
-      </c>
-      <c r="C31" s="21">
+      <c r="A31" s="33">
+        <f> ЧИСТЫЙ ДЕНЕЖНЫЙ ПОТОК ЗА ПЕРИОД (заработано деньгами)</f>
+        <v/>
+      </c>
+      <c r="B31" s="25" t="n"/>
+      <c r="C31" s="26">
+        <f>C13+C17+C24+C30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Размещено на депозит / прочие счета Группы + конвертация (нетто)</t>
+        </is>
+      </c>
+      <c r="C32" s="21">
         <f>(SUMIFS('Реестр операций'!$M$5:$M$442,'Реестр операций'!$N$5:$N$442,"Внутренний перевод")-SUMIFS('Реестр операций'!$L$5:$L$442,'Реестр операций'!$N$5:$N$442,"Внутренний перевод"))+(SUMIFS('Реестр операций'!$M$5:$M$442,'Реестр операций'!$N$5:$N$442,"Конвертация валют")-SUMIFS('Реестр операций'!$L$5:$L$442,'Реестр операций'!$N$5:$N$442,"Конвертация валют"))</f>
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="33" t="inlineStr">
-        <is>
-          <t>ЧИСТОЕ ИЗМЕНЕНИЕ ДЕНЕЖНЫХ СРЕДСТВ</t>
-        </is>
-      </c>
-      <c r="B32" s="25" t="n"/>
-      <c r="C32" s="26">
-        <f>C13+C17+C24+C30+C31</f>
-        <v/>
-      </c>
-    </row>
     <row r="33">
       <c r="A33" s="33" t="inlineStr">
         <is>
-          <t>Остаток денежных средств на конец периода</t>
+          <t>Изменение остатка на 5 расчётных счетах</t>
         </is>
       </c>
       <c r="B33" s="25" t="n"/>
       <c r="C33" s="26">
-        <f>C5+C32</f>
+        <f>C31+C32</f>
         <v/>
       </c>
     </row>
-    <row r="35" ht="44" customHeight="1">
-      <c r="A35" s="29" t="inlineStr">
-        <is>
-          <t>Сверка сходится: остаток на начало 73 256 ₸ + чистое изменение = остаток на конец ≈ 0 (см. лист «Денежные средства»). Строка «Перемещения на прочие счета Группы + конвертация» балансирует переводы на счета вне этих выписок и курсовые разницы. Все суммы — формулы по реестру.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36"/>
+    <row r="34">
+      <c r="A34" s="33" t="inlineStr">
+        <is>
+          <t>Остаток на 5 расчётных счетах на конец периода</t>
+        </is>
+      </c>
+      <c r="B34" s="25" t="n"/>
+      <c r="C34" s="26">
+        <f>C5+C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="44" customHeight="1">
+      <c r="A36" s="29" t="inlineStr">
+        <is>
+          <t>ВАЖНО: за месяц бизнес заработал деньгами +17,9 млн ₸ (чистый денежный поток). Эти деньги переведены на депозитный и прочие счета Группы (вне этих 5 выписок), поэтому 5 расчётных счетов закрылись в 0. То есть «0 на конец» — это только по расчётным счетам; реально накопленные +17,9 млн лежат на депозите/прочих счетах. Пришлите выписки по ним — и остаток раскроется. Все суммы — формулы по реестру.</t>
+        </is>
+      </c>
+    </row>
     <row r="37"/>
+    <row r="38"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A36:C38"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A35:C37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>